<commit_message>
removed 500 as such now
</commit_message>
<xml_diff>
--- a/gallabox_scenarios.xlsx
+++ b/gallabox_scenarios.xlsx
@@ -408,7 +408,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F7"/>
   <cols>
     <col min="1" max="1" width="58.83203125" customWidth="1"/>
     <col min="2" max="2" width="42.83203125" customWidth="1"/>
@@ -497,12 +497,72 @@
         <v>SHARED APIs (used by many scenarios)</v>
       </c>
       <c r="B3" t="str">
+        <v>Add address (Gallabox simple)</v>
+      </c>
+      <c r="C3" t="str">
+        <v>POST https://api.metrogini.com/api/whatsapp/address</v>
+      </c>
+      <c r="D3" t="str" xml:space="preserve">
+        <v xml:space="preserve">========== FIELD GUIDE ==========
+REQUIRED: mobile, complete_address, pincode, name, email
+OPTIONAL: none
+=================================
+How to use in Postman:
+- OPTIONAL query params are unchecked (disabled). Tick only if needed.
+- Body tab sends clean JSON (no comments).
+- Annotated body below is documentation for Gallabox (which fields are optional).
+Annotated body (docs only — do not paste comments into Body):
+{
+  "mobile": "{{mobile}}",  // REQUIRED
+  "complete_address": "A-204, Lotus Residency, Andheri West",  // REQUIRED
+  "pincode": "{{pincode}}",  // REQUIRED
+  "name": "Karthik",  // REQUIRED
+  "email": "karthik@example.com"  // REQUIRED
+}
+Gallabox: mobile + complete_address + pincode + name + email (all required). No separate set-default call. Prefer this over POST /api/user/address.
+{
+  "mobile": "9004186460",
+  "complete_address": "A-204, Lotus Residency, Andheri West",
+  "pincode": "400058",
+  "name": "Karthik",
+  "email": "karthik@example.com"
+}
+Required: mobile, complete_address, pincode, name, email
+Optional: none
+Server splits floor/landmark from complete_address and auto-sets default. Returns access_token for booking steps.</v>
+      </c>
+      <c r="E3" t="str" xml:space="preserve">
+        <v xml:space="preserve">{
+  "success": true,
+  "message": "Address added and set as default",
+  "data": {
+    "address_id": 3,
+    "is_default": true,
+    "pincode": "400058",
+    "complete_address": "A-204, Lotus Residency, Andheri West",
+    "floor": "A-204",
+    "landmark": "Lotus Residency",
+    "name": "Karthik",
+    "email": "karthik@example.com",
+    "access_token": "eyJ..."
+  }
+}</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Gallabox secret</v>
+      </c>
+    </row>
+    <row r="4" xml:space="preserve">
+      <c r="A4" t="str">
+        <v>SHARED APIs (used by many scenarios)</v>
+      </c>
+      <c r="B4" t="str">
         <v>Customer lookup by mobile</v>
       </c>
-      <c r="C3" t="str">
+      <c r="C4" t="str">
         <v>POST https://api.metrogini.com/api/whatsapp/customer/lookup</v>
       </c>
-      <c r="D3" t="str" xml:space="preserve">
+      <c r="D4" t="str" xml:space="preserve">
         <v xml:space="preserve">========== FIELD GUIDE ==========
 REQUIRED: mobile
 OPTIONAL: none
@@ -522,7 +582,7 @@
 Optional: none
 Also: GET /api/whatsapp/customer/lookup?mobile=</v>
       </c>
-      <c r="E3" t="str" xml:space="preserve">
+      <c r="E4" t="str" xml:space="preserve">
         <v xml:space="preserve">{
   "success": true,
   "message": "Customer found",
@@ -543,21 +603,21 @@
   }
 }</v>
       </c>
-      <c r="F3" t="str">
+      <c r="F4" t="str">
         <v>Gallabox secret</v>
       </c>
     </row>
-    <row r="4" xml:space="preserve">
-      <c r="A4" t="str">
+    <row r="5" xml:space="preserve">
+      <c r="A5" t="str">
         <v>SHARED APIs (used by many scenarios)</v>
       </c>
-      <c r="B4" t="str">
+      <c r="B5" t="str">
         <v>Login or register (OTP fallback)</v>
       </c>
-      <c r="C4" t="str">
+      <c r="C5" t="str">
         <v>POST https://api.metrogini.com/api/user/login-or-register</v>
       </c>
-      <c r="D4" t="str" xml:space="preserve">
+      <c r="D5" t="str" xml:space="preserve">
         <v xml:space="preserve">========== FIELD GUIDE ==========
 REQUIRED: mobile
 OPTIONAL: none
@@ -576,7 +636,7 @@
 Required: mobile
 Optional: none</v>
       </c>
-      <c r="E4" t="str" xml:space="preserve">
+      <c r="E5" t="str" xml:space="preserve">
         <v xml:space="preserve">{
   "success": true,
   "message": "OTP sent successfully",
@@ -586,21 +646,21 @@
   }
 }</v>
       </c>
-      <c r="F4" t="str">
+      <c r="F5" t="str">
         <v>No</v>
       </c>
     </row>
-    <row r="5" xml:space="preserve">
-      <c r="A5" t="str">
+    <row r="6" xml:space="preserve">
+      <c r="A6" t="str">
         <v>SHARED APIs (used by many scenarios)</v>
       </c>
-      <c r="B5" t="str">
+      <c r="B6" t="str">
         <v>Verify OTP (OTP fallback)</v>
       </c>
-      <c r="C5" t="str">
+      <c r="C6" t="str">
         <v>POST https://api.metrogini.com/api/user/verify-otp</v>
       </c>
-      <c r="D5" t="str" xml:space="preserve">
+      <c r="D6" t="str" xml:space="preserve">
         <v xml:space="preserve">========== FIELD GUIDE ==========
 REQUIRED: mobile, otp
 OPTIONAL: none
@@ -621,7 +681,7 @@
 Required: mobile, otp
 Optional: none</v>
       </c>
-      <c r="E5" t="str" xml:space="preserve">
+      <c r="E6" t="str" xml:space="preserve">
         <v xml:space="preserve">{
   "success": true,
   "data": {
@@ -631,21 +691,21 @@
   }
 }</v>
       </c>
-      <c r="F5" t="str">
+      <c r="F6" t="str">
         <v>No</v>
       </c>
     </row>
-    <row r="6" xml:space="preserve">
-      <c r="A6" t="str">
+    <row r="7" xml:space="preserve">
+      <c r="A7" t="str">
         <v>SHARED APIs (used by many scenarios)</v>
       </c>
-      <c r="B6" t="str">
+      <c r="B7" t="str">
         <v>Emit event to Gallabox (test outbound)</v>
       </c>
-      <c r="C6" t="str">
+      <c r="C7" t="str">
         <v>POST https://api.metrogini.com/api/whatsapp/events/emit</v>
       </c>
-      <c r="D6" t="str" xml:space="preserve">
+      <c r="D7" t="str" xml:space="preserve">
         <v xml:space="preserve">========== FIELD GUIDE ==========
 REQUIRED: event
 OPTIONAL: order_id, mobile, data
@@ -670,19 +730,19 @@
 Optional: order_id, mobile, data
 Events: booking_confirmed, pickup_day_reminder, rider_assigned, pickup_completed, vendor_received, weight_confirmed, order.weight_confirmed, order.finalized, payment_received, out_for_delivery, delivered, delayed, cancelled</v>
       </c>
-      <c r="E6" t="str" xml:space="preserve">
+      <c r="E7" t="str" xml:space="preserve">
         <v xml:space="preserve">{
   "success": true,
   "message": "Event queued for order"
 }</v>
       </c>
-      <c r="F6" t="str">
+      <c r="F7" t="str">
         <v>Gallabox secret</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F7"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1600,7 +1660,7 @@
   "name": "Karthik",  // REQUIRED
   "email": "karthik@example.com"  // REQUIRED
 }
-Gallabox: mobile + complete_address + pincode + name + email (all required). No separate set-default call.
+Gallabox: mobile + complete_address + pincode + name + email (all required). No separate set-default call. Prefer this over POST /api/user/address.
 {
   "mobile": "9004186460",
   "complete_address": "A-204, Lotus Residency, Andheri West",
@@ -2879,7 +2939,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <cols>
     <col min="1" max="1" width="58.83203125" customWidth="1"/>
     <col min="2" max="2" width="42.83203125" customWidth="1"/>
@@ -3026,7 +3086,8 @@
 - OPTIONAL query params are unchecked (disabled). Tick only if needed.
 - Body tab sends clean JSON (no comments).
 - Annotated body below is documentation for Gallabox (which fields are optional).
-No body. Optional: none</v>
+No body. Optional: none
+If customer picks Yes → use this address. If No → next request (WhatsApp Add address).</v>
       </c>
       <c r="E4" t="str" xml:space="preserve">
         <v xml:space="preserve">{
@@ -3051,12 +3112,72 @@
         <v>Scenario 5 — Retention: One-Time Customer, No Repeat Order</v>
       </c>
       <c r="B5" t="str">
+        <v>Change address (Gallabox simple)</v>
+      </c>
+      <c r="C5" t="str">
+        <v>POST https://api.metrogini.com/api/whatsapp/address</v>
+      </c>
+      <c r="D5" t="str" xml:space="preserve">
+        <v xml:space="preserve">========== FIELD GUIDE ==========
+REQUIRED: mobile, complete_address, pincode, name, email. Auto-sets default.
+OPTIONAL: none
+=================================
+How to use in Postman:
+- OPTIONAL query params are unchecked (disabled). Tick only if needed.
+- Body tab sends clean JSON (no comments).
+- Annotated body below is documentation for Gallabox (which fields are optional).
+Annotated body (docs only — do not paste comments into Body):
+{
+  "mobile": "{{mobile}}",  // REQUIRED
+  "complete_address": "A-204, Lotus Residency, Andheri West",  // REQUIRED
+  "pincode": "{{pincode}}",  // REQUIRED
+  "name": "Karthik",  // REQUIRED
+  "email": "karthik@example.com"  // REQUIRED
+}
+Scenario 5: customer chose No, change address. Same as Scenario 1 WhatsApp add-address. Required: mobile, complete_address, pincode, name, email. Auto-sets default.
+{
+  "mobile": "9004186460",
+  "complete_address": "A-204, Lotus Residency, Andheri West",
+  "pincode": "400058",
+  "name": "Karthik",
+  "email": "karthik@example.com"
+}
+Required: mobile, complete_address, pincode, name, email
+Optional: none
+Server splits floor/landmark from complete_address and auto-sets default. Returns access_token for booking steps.</v>
+      </c>
+      <c r="E5" t="str" xml:space="preserve">
+        <v xml:space="preserve">{
+  "success": true,
+  "message": "Address added and set as default",
+  "data": {
+    "address_id": 3,
+    "is_default": true,
+    "pincode": "400058",
+    "complete_address": "A-204, Lotus Residency, Andheri West",
+    "floor": "A-204",
+    "landmark": "Lotus Residency",
+    "name": "Karthik",
+    "email": "karthik@example.com",
+    "access_token": "eyJ..."
+  }
+}</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Gallabox secret</v>
+      </c>
+    </row>
+    <row r="6" xml:space="preserve">
+      <c r="A6" t="str">
+        <v>Scenario 5 — Retention: One-Time Customer, No Repeat Order</v>
+      </c>
+      <c r="B6" t="str">
         <v>Apply coupon (VALUED10 / win-back)</v>
       </c>
-      <c r="C5" t="str">
+      <c r="C6" t="str">
         <v>POST https://api.metrogini.com/api/user/order/:id/applyCoupon</v>
       </c>
-      <c r="D5" t="str" xml:space="preserve">
+      <c r="D6" t="str" xml:space="preserve">
         <v xml:space="preserve">========== FIELD GUIDE ==========
 REQUIRED: see body keys below
 OPTIONAL: coupon_code. Empty body {} reapplies loyalty coupon.
@@ -3076,18 +3197,18 @@
 Optional: coupon_code — omit or {} to reapply loyalty
 Txt also listed POST /api/whatsapp/offers/apply — not built; use this.</v>
       </c>
-      <c r="E5" t="str" xml:space="preserve">
+      <c r="E6" t="str" xml:space="preserve">
         <v xml:space="preserve">{
   "message": "Coupon applied successfully"
 }</v>
       </c>
-      <c r="F5" t="str">
+      <c r="F6" t="str">
         <v>Yes (user Bearer)</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F6"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>